<commit_message>
PM-Stammdaten dynamisch aus Excel-Tab 'PM-Stammdaten' geladen — kein hardcoded PMS/TOKENS mehr. Neuer PM: Zeile im Excel anhängen, Token via secrets.token_hex(16)
</commit_message>
<xml_diff>
--- a/generator/PM_Gehaltsmodell_v18.xlsx
+++ b/generator/PM_Gehaltsmodell_v18.xlsx
@@ -14,15 +14,16 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Laura" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Marleen" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Luise" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Max" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daten" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berechnung" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameter" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stufentabelle" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TH-Zulagen" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PM-Vorlage" sheetId="16" state="hidden" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kalibrierung alt" sheetId="17" state="hidden" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PM-Stammdaten" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Max" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daten" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berechnung" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameter" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stufentabelle" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TH-Zulagen" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PM-Vorlage" sheetId="17" state="hidden" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kalibrierung alt" sheetId="18" state="hidden" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -47,10 +48,10 @@
     <numFmt numFmtId="176" formatCode="#,##0.00&quot; €/h&quot;"/>
     <numFmt numFmtId="177" formatCode="\+#,##0&quot; €&quot;"/>
     <numFmt numFmtId="178" formatCode="\+#,##0.00&quot; €/h&quot;"/>
-    <numFmt numFmtId="179" formatCode="#,##0 €"/>
-    <numFmt numFmtId="180" formatCode="#,##0.0"/>
+    <numFmt numFmtId="179" formatCode="#,##0.0"/>
+    <numFmt numFmtId="180" formatCode="#,##0 €"/>
   </numFmts>
-  <fonts count="48">
+  <fonts count="50">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -348,6 +349,13 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <i val="1"/>
+    </font>
+    <font>
+      <name val="SF Mono"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="33">
@@ -649,7 +657,7 @@
     <xf numFmtId="43" fontId="24" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="24" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="156">
+  <cellXfs count="162">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1015,27 +1023,41 @@
     <xf numFmtId="0" fontId="0" fillId="31" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="179" fontId="0" fillId="31" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="180" fontId="0" fillId="31" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="4" fontId="0" fillId="31" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="32" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="32" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="180" fontId="0" fillId="32" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="32" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="179" fontId="0" fillId="31" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="0" fillId="31" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="180" fontId="0" fillId="31" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="32" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="179" fontId="0" fillId="32" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="180" fontId="0" fillId="32" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="179" fontId="0" fillId="32" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="32" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="49" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -2043,6 +2065,482 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="FFFF9800"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:F52"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" style="97" min="1" max="1"/>
+    <col width="32" customWidth="1" style="97" min="2" max="2"/>
+    <col width="26" customWidth="1" style="97" min="3" max="3"/>
+    <col width="24" customWidth="1" style="97" min="4" max="4"/>
+    <col width="20" customWidth="1" style="97" min="5" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="40" customHeight="1" s="97">
+      <c r="B1" s="106" t="inlineStr">
+        <is>
+          <t>Max — Dein Gehaltsmodell</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1" s="97">
+      <c r="B2" s="107" t="inlineStr">
+        <is>
+          <t>Deine persönliche Übersicht — Gehalt, Stufe und was du für die nächste Stufe brauchst.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="26" customHeight="1" s="97">
+      <c r="B4" s="100" t="inlineStr">
+        <is>
+          <t>1. Du und dein Bundle</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1" s="97">
+      <c r="B6" s="69" t="inlineStr">
+        <is>
+          <t>Name:</t>
+        </is>
+      </c>
+      <c r="D6" s="70">
+        <f>Daten!B8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1" s="97">
+      <c r="B7" s="69" t="inlineStr">
+        <is>
+          <t>Dein Bundle:</t>
+        </is>
+      </c>
+      <c r="D7" s="70" t="inlineStr">
+        <is>
+          <t>Spandau, Mitte</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1" s="97">
+      <c r="B8" s="69" t="inlineStr">
+        <is>
+          <t>Wochenstunden:</t>
+        </is>
+      </c>
+      <c r="D8" s="114">
+        <f>Daten!C8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1" s="97">
+      <c r="B9" s="69" t="inlineStr">
+        <is>
+          <t>Startdatum:</t>
+        </is>
+      </c>
+      <c r="D9" s="70">
+        <f>IFERROR(TEXT(Daten!A8,"DD.MM.YYYY"),"(seit Anfang)")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1" s="97">
+      <c r="B10" s="69" t="inlineStr">
+        <is>
+          <t>Mindestgehalt pro Jahr:</t>
+        </is>
+      </c>
+      <c r="D10" s="72">
+        <f>Daten!F8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="26" customHeight="1" s="97">
+      <c r="B13" s="100" t="inlineStr">
+        <is>
+          <t>2. Dein aktuelles Gehalt (letztes abgeschlossenes Quartal: Q1 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="36" customHeight="1" s="97">
+      <c r="B15" s="69" t="inlineStr">
+        <is>
+          <t>Dein Monatsgehalt (ab Q2 2026):</t>
+        </is>
+      </c>
+      <c r="D15" s="73">
+        <f>IFERROR(Berechnung!T8,"(fehlt Zufr-Wert)")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1" s="97">
+      <c r="B16" s="69" t="inlineStr">
+        <is>
+          <t>Stufe:</t>
+        </is>
+      </c>
+      <c r="D16" s="70">
+        <f>IFERROR(Berechnung!O8 &amp; " - " &amp; Berechnung!P8,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1" s="97">
+      <c r="B17" s="69" t="inlineStr">
+        <is>
+          <t>Jahresgehalt:</t>
+        </is>
+      </c>
+      <c r="D17" s="72">
+        <f>IFERROR(Berechnung!S8,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="26" customHeight="1" s="97">
+      <c r="B19" s="100" t="inlineStr">
+        <is>
+          <t>3. Warum diese Stufe?</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1" s="97">
+      <c r="B21" s="69" t="inlineStr">
+        <is>
+          <t>Dein Leistungsindex (€/60min Therapie):</t>
+        </is>
+      </c>
+      <c r="D21" s="115">
+        <f>IFERROR(Daten!J8/(Daten!H8-Daten!I8),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="24" customHeight="1" s="97">
+      <c r="B22" s="69" t="inlineStr">
+        <is>
+          <t>Deine Team-Zufriedenheit (0-10):</t>
+        </is>
+      </c>
+      <c r="D22" s="75">
+        <f>IFERROR(Berechnung!C8,"(fehlt Umfrage-Wert)")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="28" customHeight="1" s="97">
+      <c r="B24" s="102" t="inlineStr">
+        <is>
+          <t>Deine erreichte Stufe ergibt sich, wenn BEIDE Werte oben den Schwellen entsprechen (siehe Modell-Tab).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="26" customHeight="1" s="97">
+      <c r="B26" s="100" t="inlineStr">
+        <is>
+          <t>4. Was bringt dir die nächste Stufe?</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="24" customHeight="1" s="97">
+      <c r="B28" s="69" t="inlineStr">
+        <is>
+          <t>Nächste erreichbare Stufe:</t>
+        </is>
+      </c>
+      <c r="D28" s="76">
+        <f>IFERROR((IF(IFERROR(Berechnung!O8,0)&lt;6,IFERROR(Berechnung!O8,0)+1,6)) &amp; " - " &amp; INDEX({"Basis";"Gut";"Stark";"Sehr stark";"Exzellent";"Herausragend"},IF(IFERROR(Berechnung!O8,0)&lt;6,IFERROR(Berechnung!O8,0)+1,6)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" ht="32" customHeight="1" s="97">
+      <c r="B29" s="69" t="inlineStr">
+        <is>
+          <t>Mehr pro Monat (Δ):</t>
+        </is>
+      </c>
+      <c r="D29" s="116">
+        <f>IFERROR(Berechnung!T8*((IFERROR(INDEX(Stufentabelle!E2:E7,IF(IFERROR(Berechnung!O8,0)&lt;6,IFERROR(Berechnung!O8,0)+1,6)),0))-(IFERROR(INDEX(Stufentabelle!E2:E7,Berechnung!O8),0)))/(1+(IFERROR(INDEX(Stufentabelle!E2:E7,Berechnung!O8),0))),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" ht="24" customHeight="1" s="97">
+      <c r="B30" s="69" t="inlineStr">
+        <is>
+          <t>Mehr pro Jahr (Δ):</t>
+        </is>
+      </c>
+      <c r="D30" s="117">
+        <f>IFERROR(Berechnung!S8*((IFERROR(INDEX(Stufentabelle!E2:E7,IF(IFERROR(Berechnung!O8,0)&lt;6,IFERROR(Berechnung!O8,0)+1,6)),0))-(IFERROR(INDEX(Stufentabelle!E2:E7,Berechnung!O8),0)))/(1+(IFERROR(INDEX(Stufentabelle!E2:E7,Berechnung!O8),0))),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" ht="26" customHeight="1" s="97">
+      <c r="B32" s="100" t="inlineStr">
+        <is>
+          <t>5. Was fehlt dir für die nächste Stufe?</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="24" customHeight="1" s="97">
+      <c r="B34" s="69" t="inlineStr">
+        <is>
+          <t>Zielwert €/60min:</t>
+        </is>
+      </c>
+      <c r="D34" s="118">
+        <f>IFERROR(INDEX(Stufentabelle!F2:F7,IF(IFERROR(Berechnung!O8,0)&lt;6,IFERROR(Berechnung!O8,0)+1,6)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" ht="24" customHeight="1" s="97">
+      <c r="B35" s="69" t="inlineStr">
+        <is>
+          <t>Fehlt dir pro Therapie-Stunde:</t>
+        </is>
+      </c>
+      <c r="D35" s="119">
+        <f>IFERROR(MAX(0,(INDEX(Stufentabelle!F2:F7,IF(IFERROR(Berechnung!O8,0)&lt;6,IFERROR(Berechnung!O8,0)+1,6)))-(Daten!J8/(Daten!H8-Daten!I8))),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" ht="32" customHeight="1" s="97">
+      <c r="B36" s="69" t="inlineStr">
+        <is>
+          <t>In Bundle-Umsatz pro Monat:</t>
+        </is>
+      </c>
+      <c r="D36" s="120">
+        <f>IFERROR(MAX(0,((INDEX(Stufentabelle!F2:F7,IF(IFERROR(Berechnung!O8,0)&lt;6,IFERROR(Berechnung!O8,0)+1,6)))*(Daten!H8-Daten!I8)-Daten!J8)/3),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" ht="26" customHeight="1" s="97">
+      <c r="B38" s="100" t="inlineStr">
+        <is>
+          <t>6. Hebel — so schaffst du das</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="20" customHeight="1" s="97">
+      <c r="B39" s="102" t="inlineStr">
+        <is>
+          <t>Hinweis: Effekte sind Orientierungswerte (grobe Rechnung), keine exakten Prognosen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="30" customHeight="1" s="97">
+      <c r="B40" s="57" t="inlineStr">
+        <is>
+          <t>Hebel</t>
+        </is>
+      </c>
+      <c r="C40" s="57" t="inlineStr">
+        <is>
+          <t>Effekt</t>
+        </is>
+      </c>
+      <c r="D40" s="57" t="inlineStr">
+        <is>
+          <t>Praktisch</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="30" customHeight="1" s="97">
+      <c r="B41" s="82" t="inlineStr">
+        <is>
+          <t>Mehr Termine pro Woche</t>
+        </is>
+      </c>
+      <c r="C41" s="82" t="inlineStr">
+        <is>
+          <t>+10 Termine/Wo ≈ +3 % Umsatz</t>
+        </is>
+      </c>
+      <c r="D41" s="82" t="inlineStr">
+        <is>
+          <t>Auslastung hoch, Neukunden, Slots besser nutzen</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="30" customHeight="1" s="97">
+      <c r="B42" s="83" t="inlineStr">
+        <is>
+          <t>Mehr PKV-Anteil</t>
+        </is>
+      </c>
+      <c r="C42" s="83" t="inlineStr">
+        <is>
+          <t>+1 %-Pkt PKV ≈ +0,7 % Umsatz</t>
+        </is>
+      </c>
+      <c r="D42" s="83" t="inlineStr">
+        <is>
+          <t>Privatpatienten aktiv gewinnen (1,7× Tarif)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="30" customHeight="1" s="97">
+      <c r="B43" s="82" t="inlineStr">
+        <is>
+          <t>Weniger Krankenstand</t>
+        </is>
+      </c>
+      <c r="C43" s="82" t="inlineStr">
+        <is>
+          <t>−1 %-Pkt Krank ≈ +0,5 % Umsatz</t>
+        </is>
+      </c>
+      <c r="D43" s="82" t="inlineStr">
+        <is>
+          <t>Team-Gesundheit, gute Urlaubsplanung</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="26" customHeight="1" s="97">
+      <c r="B46" s="100" t="inlineStr">
+        <is>
+          <t>7. Deine Entwicklung über die Quartale</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="22" customHeight="1" s="97">
+      <c r="B48" s="57" t="inlineStr">
+        <is>
+          <t>Quartal</t>
+        </is>
+      </c>
+      <c r="C48" s="57" t="inlineStr">
+        <is>
+          <t>Stufe</t>
+        </is>
+      </c>
+      <c r="D48" s="57" t="inlineStr">
+        <is>
+          <t>€/60min</t>
+        </is>
+      </c>
+      <c r="E48" s="57" t="inlineStr">
+        <is>
+          <t>Monatsgehalt</t>
+        </is>
+      </c>
+      <c r="F48" s="57" t="inlineStr">
+        <is>
+          <t>Jahresgehalt</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="22" customHeight="1" s="97">
+      <c r="B49" s="70" t="inlineStr">
+        <is>
+          <t>Q1 2026</t>
+        </is>
+      </c>
+      <c r="C49" s="84">
+        <f>IFERROR(Berechnung!O8 &amp; " - " &amp; Berechnung!P8,"-")</f>
+        <v/>
+      </c>
+      <c r="D49" s="121">
+        <f>IFERROR(Daten!J8/(Daten!H8-Daten!I8),"-")</f>
+        <v/>
+      </c>
+      <c r="E49" s="86">
+        <f>IFERROR(Berechnung!T8,"-")</f>
+        <v/>
+      </c>
+      <c r="F49" s="86">
+        <f>IFERROR(Berechnung!S8,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" ht="22" customHeight="1" s="97">
+      <c r="B50" s="70" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="C50" s="84">
+        <f>IFERROR(Berechnung!AG8 &amp; " - " &amp; Berechnung!AH8,"-")</f>
+        <v/>
+      </c>
+      <c r="D50" s="121">
+        <f>IFERROR(Daten!Q8/(Daten!O8-Daten!P8),"-")</f>
+        <v/>
+      </c>
+      <c r="E50" s="86">
+        <f>IFERROR(Berechnung!AL8,"-")</f>
+        <v/>
+      </c>
+      <c r="F50" s="86">
+        <f>IFERROR(Berechnung!AK8,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51" ht="22" customHeight="1" s="97">
+      <c r="B51" s="70" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="C51" s="84">
+        <f>IFERROR(Berechnung!AY8 &amp; " - " &amp; Berechnung!AZ8,"-")</f>
+        <v/>
+      </c>
+      <c r="D51" s="121">
+        <f>IFERROR(Daten!X8/(Daten!V8-Daten!W8),"-")</f>
+        <v/>
+      </c>
+      <c r="E51" s="86">
+        <f>IFERROR(Berechnung!BD8,"-")</f>
+        <v/>
+      </c>
+      <c r="F51" s="86">
+        <f>IFERROR(Berechnung!BC8,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52" ht="22" customHeight="1" s="97">
+      <c r="B52" s="70" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="C52" s="84">
+        <f>IFERROR(Berechnung!BQ8 &amp; " - " &amp; Berechnung!BR8,"-")</f>
+        <v/>
+      </c>
+      <c r="D52" s="121">
+        <f>IFERROR(Daten!AE8/(Daten!AC8-Daten!AD8),"-")</f>
+        <v/>
+      </c>
+      <c r="E52" s="86">
+        <f>IFERROR(Berechnung!BV8,"-")</f>
+        <v/>
+      </c>
+      <c r="F52" s="86">
+        <f>IFERROR(Berechnung!BU8,"-")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="B39:F39"/>
+    <mergeCell ref="B24:F24"/>
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="B38:F38"/>
+    <mergeCell ref="B19:F19"/>
+    <mergeCell ref="B46:F46"/>
+    <mergeCell ref="B1:F1"/>
+    <mergeCell ref="B32:F32"/>
+    <mergeCell ref="B26:F26"/>
+    <mergeCell ref="B13:F13"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -2316,7 +2814,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3566,7 +4064,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FFBDBDBD"/>
@@ -6413,7 +6911,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FFBDBDBD"/>
@@ -6514,14 +7012,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FFBDBDBD"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="8" customWidth="1" style="97" min="1" max="1"/>
@@ -6644,8 +7142,6 @@
         <v>89.48</v>
       </c>
     </row>
-    <row r="8"/>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="113" t="inlineStr">
         <is>
@@ -6664,7 +7160,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FFBDBDBD"/>
@@ -7063,7 +7559,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FFBDBDBD"/>
@@ -7085,7 +7581,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8147,24 +8643,24 @@
           <t>Spandau, Mitte</t>
         </is>
       </c>
-      <c r="C8" s="149" t="n">
+      <c r="C8" s="156" t="n">
         <v>4924</v>
       </c>
-      <c r="D8" s="149" t="n">
+      <c r="D8" s="156" t="n">
         <v>4686.3</v>
       </c>
-      <c r="E8" s="149" t="n">
+      <c r="E8" s="156" t="n">
         <v>554.8</v>
       </c>
-      <c r="F8" s="149" t="inlineStr">
+      <c r="F8" s="156" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G8" s="150" t="n">
+      <c r="G8" s="157" t="n">
         <v>291941</v>
       </c>
-      <c r="H8" s="149" t="n">
+      <c r="H8" s="156" t="n">
         <v>4131.5</v>
       </c>
       <c r="I8" s="151" t="n">
@@ -8211,24 +8707,24 @@
           <t>Friedrichshain, Charlottenburg, Prenzlauer Berg</t>
         </is>
       </c>
-      <c r="C9" s="149" t="n">
+      <c r="C9" s="156" t="n">
         <v>5665.2</v>
       </c>
-      <c r="D9" s="149" t="n">
+      <c r="D9" s="156" t="n">
         <v>5343.5</v>
       </c>
-      <c r="E9" s="149" t="n">
+      <c r="E9" s="156" t="n">
         <v>293.5</v>
       </c>
-      <c r="F9" s="149" t="inlineStr">
+      <c r="F9" s="156" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G9" s="150" t="n">
+      <c r="G9" s="157" t="n">
         <v>337924</v>
       </c>
-      <c r="H9" s="149" t="n">
+      <c r="H9" s="156" t="n">
         <v>5050</v>
       </c>
       <c r="I9" s="151" t="n">
@@ -8275,24 +8771,24 @@
           <t>Friedrichshain, Charlottenburg, Prenzlauer Berg</t>
         </is>
       </c>
-      <c r="C10" s="149" t="n">
+      <c r="C10" s="156" t="n">
         <v>5665.2</v>
       </c>
-      <c r="D10" s="149" t="n">
+      <c r="D10" s="156" t="n">
         <v>5343.5</v>
       </c>
-      <c r="E10" s="149" t="n">
+      <c r="E10" s="156" t="n">
         <v>293.5</v>
       </c>
-      <c r="F10" s="149" t="inlineStr">
+      <c r="F10" s="156" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G10" s="150" t="n">
+      <c r="G10" s="157" t="n">
         <v>337924</v>
       </c>
-      <c r="H10" s="149" t="n">
+      <c r="H10" s="156" t="n">
         <v>5050</v>
       </c>
       <c r="I10" s="151" t="n">
@@ -8339,24 +8835,24 @@
           <t>Spandau, Mitte</t>
         </is>
       </c>
-      <c r="C11" s="149" t="n">
+      <c r="C11" s="156" t="n">
         <v>4924</v>
       </c>
-      <c r="D11" s="149" t="n">
+      <c r="D11" s="156" t="n">
         <v>4686.3</v>
       </c>
-      <c r="E11" s="149" t="n">
+      <c r="E11" s="156" t="n">
         <v>554.8</v>
       </c>
-      <c r="F11" s="149" t="inlineStr">
+      <c r="F11" s="156" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G11" s="150" t="n">
+      <c r="G11" s="157" t="n">
         <v>291941</v>
       </c>
-      <c r="H11" s="149" t="n">
+      <c r="H11" s="156" t="n">
         <v>4131.5</v>
       </c>
       <c r="I11" s="151" t="n">
@@ -8542,12 +9038,12 @@
           <t>Spandau, Mitte</t>
         </is>
       </c>
-      <c r="C8" s="153" t="inlineStr"/>
-      <c r="D8" s="153" t="inlineStr"/>
-      <c r="E8" s="153" t="inlineStr"/>
-      <c r="F8" s="153" t="inlineStr"/>
-      <c r="G8" s="154" t="inlineStr"/>
-      <c r="H8" s="153" t="inlineStr"/>
+      <c r="C8" s="158" t="inlineStr"/>
+      <c r="D8" s="158" t="inlineStr"/>
+      <c r="E8" s="158" t="inlineStr"/>
+      <c r="F8" s="158" t="inlineStr"/>
+      <c r="G8" s="159" t="inlineStr"/>
+      <c r="H8" s="158" t="inlineStr"/>
       <c r="I8" s="155" t="inlineStr"/>
       <c r="J8" s="155" t="inlineStr"/>
       <c r="K8" s="152" t="inlineStr"/>
@@ -8572,12 +9068,12 @@
           <t>Friedrichshain, Charlottenburg, Prenzlauer Berg</t>
         </is>
       </c>
-      <c r="C9" s="153" t="inlineStr"/>
-      <c r="D9" s="153" t="inlineStr"/>
-      <c r="E9" s="153" t="inlineStr"/>
-      <c r="F9" s="153" t="inlineStr"/>
-      <c r="G9" s="154" t="inlineStr"/>
-      <c r="H9" s="153" t="inlineStr"/>
+      <c r="C9" s="158" t="inlineStr"/>
+      <c r="D9" s="158" t="inlineStr"/>
+      <c r="E9" s="158" t="inlineStr"/>
+      <c r="F9" s="158" t="inlineStr"/>
+      <c r="G9" s="159" t="inlineStr"/>
+      <c r="H9" s="158" t="inlineStr"/>
       <c r="I9" s="155" t="inlineStr"/>
       <c r="J9" s="155" t="inlineStr"/>
       <c r="K9" s="152" t="inlineStr"/>
@@ -8602,12 +9098,12 @@
           <t>Friedrichshain, Charlottenburg, Prenzlauer Berg</t>
         </is>
       </c>
-      <c r="C10" s="153" t="inlineStr"/>
-      <c r="D10" s="153" t="inlineStr"/>
-      <c r="E10" s="153" t="inlineStr"/>
-      <c r="F10" s="153" t="inlineStr"/>
-      <c r="G10" s="154" t="inlineStr"/>
-      <c r="H10" s="153" t="inlineStr"/>
+      <c r="C10" s="158" t="inlineStr"/>
+      <c r="D10" s="158" t="inlineStr"/>
+      <c r="E10" s="158" t="inlineStr"/>
+      <c r="F10" s="158" t="inlineStr"/>
+      <c r="G10" s="159" t="inlineStr"/>
+      <c r="H10" s="158" t="inlineStr"/>
       <c r="I10" s="155" t="inlineStr"/>
       <c r="J10" s="155" t="inlineStr"/>
       <c r="K10" s="152" t="inlineStr"/>
@@ -8632,12 +9128,12 @@
           <t>Spandau, Mitte</t>
         </is>
       </c>
-      <c r="C11" s="153" t="inlineStr"/>
-      <c r="D11" s="153" t="inlineStr"/>
-      <c r="E11" s="153" t="inlineStr"/>
-      <c r="F11" s="153" t="inlineStr"/>
-      <c r="G11" s="154" t="inlineStr"/>
-      <c r="H11" s="153" t="inlineStr"/>
+      <c r="C11" s="158" t="inlineStr"/>
+      <c r="D11" s="158" t="inlineStr"/>
+      <c r="E11" s="158" t="inlineStr"/>
+      <c r="F11" s="158" t="inlineStr"/>
+      <c r="G11" s="159" t="inlineStr"/>
+      <c r="H11" s="158" t="inlineStr"/>
       <c r="I11" s="155" t="inlineStr"/>
       <c r="J11" s="155" t="inlineStr"/>
       <c r="K11" s="152" t="inlineStr"/>
@@ -10215,474 +10711,277 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="FFFF9800"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:F52"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <dimension ref="A1:J12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="2" customWidth="1" style="97" min="1" max="1"/>
-    <col width="32" customWidth="1" style="97" min="2" max="2"/>
-    <col width="26" customWidth="1" style="97" min="3" max="3"/>
-    <col width="24" customWidth="1" style="97" min="4" max="4"/>
-    <col width="20" customWidth="1" style="97" min="5" max="6"/>
+    <col width="10" customWidth="1" style="97" min="1" max="1"/>
+    <col width="10" customWidth="1" style="97" min="2" max="2"/>
+    <col width="12" customWidth="1" style="97" min="3" max="3"/>
+    <col width="12" customWidth="1" style="97" min="4" max="4"/>
+    <col width="14" customWidth="1" style="97" min="5" max="5"/>
+    <col width="35" customWidth="1" style="97" min="6" max="6"/>
+    <col width="18" customWidth="1" style="97" min="7" max="7"/>
+    <col width="12" customWidth="1" style="97" min="8" max="8"/>
+    <col width="35" customWidth="1" style="97" min="9" max="9"/>
+    <col width="8" customWidth="1" style="97" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1" s="97">
-      <c r="B1" s="106" t="inlineStr">
-        <is>
-          <t>Max — Dein Gehaltsmodell</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="22" customHeight="1" s="97">
-      <c r="B2" s="107" t="inlineStr">
-        <is>
-          <t>Deine persönliche Übersicht — Gehalt, Stufe und was du für die nächste Stufe brauchst.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="26" customHeight="1" s="97">
-      <c r="B4" s="100" t="inlineStr">
-        <is>
-          <t>1. Du und dein Bundle</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="22" customHeight="1" s="97">
-      <c r="B6" s="69" t="inlineStr">
-        <is>
-          <t>Name:</t>
-        </is>
-      </c>
-      <c r="D6" s="70">
-        <f>Daten!B8</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1" s="97">
-      <c r="B7" s="69" t="inlineStr">
-        <is>
-          <t>Dein Bundle:</t>
-        </is>
-      </c>
-      <c r="D7" s="70" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="136" t="inlineStr">
+        <is>
+          <t>👥 PM-Stammdaten (Quelle der Wahrheit für PM-Liste)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="50" customHeight="1" s="97">
+      <c r="A3" s="137" t="inlineStr">
+        <is>
+          <t>Code liest beim Start dieses Sheet, NICHT mehr eine hardcoded Liste. Neuen PM hinzufügen: einfach neue Zeile anhängen, Token via python3 -c "import secrets; print(secrets.token_hex(16))" erzeugen, Daten-Tab Q-Spalten parallel anlegen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1" s="97">
+      <c r="A5" s="147" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B5" s="147" t="inlineStr">
+        <is>
+          <t>Wochenstd</t>
+        </is>
+      </c>
+      <c r="C5" s="147" t="inlineStr">
+        <is>
+          <t>PM-Std Bundle</t>
+        </is>
+      </c>
+      <c r="D5" s="147" t="inlineStr">
+        <is>
+          <t>Mindestgehalt</t>
+        </is>
+      </c>
+      <c r="E5" s="147" t="inlineStr">
+        <is>
+          <t>Startdatum</t>
+        </is>
+      </c>
+      <c r="F5" s="147" t="inlineStr">
+        <is>
+          <t>Bundle-Standorte</t>
+        </is>
+      </c>
+      <c r="G5" s="147" t="inlineStr">
+        <is>
+          <t>Bundle-PMs</t>
+        </is>
+      </c>
+      <c r="H5" s="147" t="inlineStr">
+        <is>
+          <t>Farbe (Hex)</t>
+        </is>
+      </c>
+      <c r="I5" s="147" t="inlineStr">
+        <is>
+          <t>URL-Token (32-hex)</t>
+        </is>
+      </c>
+      <c r="J5" s="147" t="inlineStr">
+        <is>
+          <t>Aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="137" t="inlineStr">
+        <is>
+          <t>Laura</t>
+        </is>
+      </c>
+      <c r="B6" s="137" t="n">
+        <v>40</v>
+      </c>
+      <c r="C6" s="137" t="n">
+        <v>65</v>
+      </c>
+      <c r="D6" s="137" t="n">
+        <v>45000</v>
+      </c>
+      <c r="E6" s="137" t="n"/>
+      <c r="F6" s="137" t="inlineStr">
         <is>
           <t>Spandau, Mitte</t>
         </is>
       </c>
-    </row>
-    <row r="8" ht="22" customHeight="1" s="97">
-      <c r="B8" s="69" t="inlineStr">
-        <is>
-          <t>Wochenstunden:</t>
-        </is>
-      </c>
-      <c r="D8" s="114">
-        <f>Daten!C8</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1" s="97">
-      <c r="B9" s="69" t="inlineStr">
-        <is>
-          <t>Startdatum:</t>
-        </is>
-      </c>
-      <c r="D9" s="70">
-        <f>IFERROR(TEXT(Daten!A8,"DD.MM.YYYY"),"(seit Anfang)")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10" ht="22" customHeight="1" s="97">
-      <c r="B10" s="69" t="inlineStr">
-        <is>
-          <t>Mindestgehalt pro Jahr:</t>
-        </is>
-      </c>
-      <c r="D10" s="72">
-        <f>Daten!F8</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13" ht="26" customHeight="1" s="97">
-      <c r="B13" s="100" t="inlineStr">
-        <is>
-          <t>2. Dein aktuelles Gehalt (letztes abgeschlossenes Quartal: Q1 2026)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="36" customHeight="1" s="97">
-      <c r="B15" s="69" t="inlineStr">
-        <is>
-          <t>Dein Monatsgehalt (ab Q2 2026):</t>
-        </is>
-      </c>
-      <c r="D15" s="73">
-        <f>IFERROR(Berechnung!T8,"(fehlt Zufr-Wert)")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16" ht="24" customHeight="1" s="97">
-      <c r="B16" s="69" t="inlineStr">
-        <is>
-          <t>Stufe:</t>
-        </is>
-      </c>
-      <c r="D16" s="70">
-        <f>IFERROR(Berechnung!O8 &amp; " - " &amp; Berechnung!P8,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" ht="24" customHeight="1" s="97">
-      <c r="B17" s="69" t="inlineStr">
-        <is>
-          <t>Jahresgehalt:</t>
-        </is>
-      </c>
-      <c r="D17" s="72">
-        <f>IFERROR(Berechnung!S8,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19" ht="26" customHeight="1" s="97">
-      <c r="B19" s="100" t="inlineStr">
-        <is>
-          <t>3. Warum diese Stufe?</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="30" customHeight="1" s="97">
-      <c r="B21" s="69" t="inlineStr">
-        <is>
-          <t>Dein Leistungsindex (€/60min Therapie):</t>
-        </is>
-      </c>
-      <c r="D21" s="115">
-        <f>IFERROR(Daten!J8/(Daten!H8-Daten!I8),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22" ht="24" customHeight="1" s="97">
-      <c r="B22" s="69" t="inlineStr">
-        <is>
-          <t>Deine Team-Zufriedenheit (0-10):</t>
-        </is>
-      </c>
-      <c r="D22" s="75">
-        <f>IFERROR(Berechnung!C8,"(fehlt Umfrage-Wert)")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24" ht="28" customHeight="1" s="97">
-      <c r="B24" s="102" t="inlineStr">
-        <is>
-          <t>Deine erreichte Stufe ergibt sich, wenn BEIDE Werte oben den Schwellen entsprechen (siehe Modell-Tab).</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="26" customHeight="1" s="97">
-      <c r="B26" s="100" t="inlineStr">
-        <is>
-          <t>4. Was bringt dir die nächste Stufe?</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="24" customHeight="1" s="97">
-      <c r="B28" s="69" t="inlineStr">
-        <is>
-          <t>Nächste erreichbare Stufe:</t>
-        </is>
-      </c>
-      <c r="D28" s="76">
-        <f>IFERROR((IF(IFERROR(Berechnung!O8,0)&lt;6,IFERROR(Berechnung!O8,0)+1,6)) &amp; " - " &amp; INDEX({"Basis";"Gut";"Stark";"Sehr stark";"Exzellent";"Herausragend"},IF(IFERROR(Berechnung!O8,0)&lt;6,IFERROR(Berechnung!O8,0)+1,6)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29" ht="32" customHeight="1" s="97">
-      <c r="B29" s="69" t="inlineStr">
-        <is>
-          <t>Mehr pro Monat (Δ):</t>
-        </is>
-      </c>
-      <c r="D29" s="116">
-        <f>IFERROR(Berechnung!T8*((IFERROR(INDEX(Stufentabelle!E2:E7,IF(IFERROR(Berechnung!O8,0)&lt;6,IFERROR(Berechnung!O8,0)+1,6)),0))-(IFERROR(INDEX(Stufentabelle!E2:E7,Berechnung!O8),0)))/(1+(IFERROR(INDEX(Stufentabelle!E2:E7,Berechnung!O8),0))),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30" ht="24" customHeight="1" s="97">
-      <c r="B30" s="69" t="inlineStr">
-        <is>
-          <t>Mehr pro Jahr (Δ):</t>
-        </is>
-      </c>
-      <c r="D30" s="117">
-        <f>IFERROR(Berechnung!S8*((IFERROR(INDEX(Stufentabelle!E2:E7,IF(IFERROR(Berechnung!O8,0)&lt;6,IFERROR(Berechnung!O8,0)+1,6)),0))-(IFERROR(INDEX(Stufentabelle!E2:E7,Berechnung!O8),0)))/(1+(IFERROR(INDEX(Stufentabelle!E2:E7,Berechnung!O8),0))),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32" ht="26" customHeight="1" s="97">
-      <c r="B32" s="100" t="inlineStr">
-        <is>
-          <t>5. Was fehlt dir für die nächste Stufe?</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="24" customHeight="1" s="97">
-      <c r="B34" s="69" t="inlineStr">
-        <is>
-          <t>Zielwert €/60min:</t>
-        </is>
-      </c>
-      <c r="D34" s="118">
-        <f>IFERROR(INDEX(Stufentabelle!F2:F7,IF(IFERROR(Berechnung!O8,0)&lt;6,IFERROR(Berechnung!O8,0)+1,6)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35" ht="24" customHeight="1" s="97">
-      <c r="B35" s="69" t="inlineStr">
-        <is>
-          <t>Fehlt dir pro Therapie-Stunde:</t>
-        </is>
-      </c>
-      <c r="D35" s="119">
-        <f>IFERROR(MAX(0,(INDEX(Stufentabelle!F2:F7,IF(IFERROR(Berechnung!O8,0)&lt;6,IFERROR(Berechnung!O8,0)+1,6)))-(Daten!J8/(Daten!H8-Daten!I8))),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36" ht="32" customHeight="1" s="97">
-      <c r="B36" s="69" t="inlineStr">
-        <is>
-          <t>In Bundle-Umsatz pro Monat:</t>
-        </is>
-      </c>
-      <c r="D36" s="120">
-        <f>IFERROR(MAX(0,((INDEX(Stufentabelle!F2:F7,IF(IFERROR(Berechnung!O8,0)&lt;6,IFERROR(Berechnung!O8,0)+1,6)))*(Daten!H8-Daten!I8)-Daten!J8)/3),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38" ht="26" customHeight="1" s="97">
-      <c r="B38" s="100" t="inlineStr">
-        <is>
-          <t>6. Hebel — so schaffst du das</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="20" customHeight="1" s="97">
-      <c r="B39" s="102" t="inlineStr">
-        <is>
-          <t>Hinweis: Effekte sind Orientierungswerte (grobe Rechnung), keine exakten Prognosen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="30" customHeight="1" s="97">
-      <c r="B40" s="57" t="inlineStr">
-        <is>
-          <t>Hebel</t>
-        </is>
-      </c>
-      <c r="C40" s="57" t="inlineStr">
-        <is>
-          <t>Effekt</t>
-        </is>
-      </c>
-      <c r="D40" s="57" t="inlineStr">
-        <is>
-          <t>Praktisch</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="30" customHeight="1" s="97">
-      <c r="B41" s="82" t="inlineStr">
-        <is>
-          <t>Mehr Termine pro Woche</t>
-        </is>
-      </c>
-      <c r="C41" s="82" t="inlineStr">
-        <is>
-          <t>+10 Termine/Wo ≈ +3 % Umsatz</t>
-        </is>
-      </c>
-      <c r="D41" s="82" t="inlineStr">
-        <is>
-          <t>Auslastung hoch, Neukunden, Slots besser nutzen</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="30" customHeight="1" s="97">
-      <c r="B42" s="83" t="inlineStr">
-        <is>
-          <t>Mehr PKV-Anteil</t>
-        </is>
-      </c>
-      <c r="C42" s="83" t="inlineStr">
-        <is>
-          <t>+1 %-Pkt PKV ≈ +0,7 % Umsatz</t>
-        </is>
-      </c>
-      <c r="D42" s="83" t="inlineStr">
-        <is>
-          <t>Privatpatienten aktiv gewinnen (1,7× Tarif)</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="30" customHeight="1" s="97">
-      <c r="B43" s="82" t="inlineStr">
-        <is>
-          <t>Weniger Krankenstand</t>
-        </is>
-      </c>
-      <c r="C43" s="82" t="inlineStr">
-        <is>
-          <t>−1 %-Pkt Krank ≈ +0,5 % Umsatz</t>
-        </is>
-      </c>
-      <c r="D43" s="82" t="inlineStr">
-        <is>
-          <t>Team-Gesundheit, gute Urlaubsplanung</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="26" customHeight="1" s="97">
-      <c r="B46" s="100" t="inlineStr">
-        <is>
-          <t>7. Deine Entwicklung über die Quartale</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="22" customHeight="1" s="97">
-      <c r="B48" s="57" t="inlineStr">
-        <is>
-          <t>Quartal</t>
-        </is>
-      </c>
-      <c r="C48" s="57" t="inlineStr">
-        <is>
-          <t>Stufe</t>
-        </is>
-      </c>
-      <c r="D48" s="57" t="inlineStr">
-        <is>
-          <t>€/60min</t>
-        </is>
-      </c>
-      <c r="E48" s="57" t="inlineStr">
-        <is>
-          <t>Monatsgehalt</t>
-        </is>
-      </c>
-      <c r="F48" s="57" t="inlineStr">
-        <is>
-          <t>Jahresgehalt</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="22" customHeight="1" s="97">
-      <c r="B49" s="70" t="inlineStr">
-        <is>
-          <t>Q1 2026</t>
-        </is>
-      </c>
-      <c r="C49" s="84">
-        <f>IFERROR(Berechnung!O8 &amp; " - " &amp; Berechnung!P8,"-")</f>
-        <v/>
-      </c>
-      <c r="D49" s="121">
-        <f>IFERROR(Daten!J8/(Daten!H8-Daten!I8),"-")</f>
-        <v/>
-      </c>
-      <c r="E49" s="86">
-        <f>IFERROR(Berechnung!T8,"-")</f>
-        <v/>
-      </c>
-      <c r="F49" s="86">
-        <f>IFERROR(Berechnung!S8,"-")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50" ht="22" customHeight="1" s="97">
-      <c r="B50" s="70" t="inlineStr">
-        <is>
-          <t>Q2 2026</t>
-        </is>
-      </c>
-      <c r="C50" s="84">
-        <f>IFERROR(Berechnung!AG8 &amp; " - " &amp; Berechnung!AH8,"-")</f>
-        <v/>
-      </c>
-      <c r="D50" s="121">
-        <f>IFERROR(Daten!Q8/(Daten!O8-Daten!P8),"-")</f>
-        <v/>
-      </c>
-      <c r="E50" s="86">
-        <f>IFERROR(Berechnung!AL8,"-")</f>
-        <v/>
-      </c>
-      <c r="F50" s="86">
-        <f>IFERROR(Berechnung!AK8,"-")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51" ht="22" customHeight="1" s="97">
-      <c r="B51" s="70" t="inlineStr">
-        <is>
-          <t>Q3 2026</t>
-        </is>
-      </c>
-      <c r="C51" s="84">
-        <f>IFERROR(Berechnung!AY8 &amp; " - " &amp; Berechnung!AZ8,"-")</f>
-        <v/>
-      </c>
-      <c r="D51" s="121">
-        <f>IFERROR(Daten!X8/(Daten!V8-Daten!W8),"-")</f>
-        <v/>
-      </c>
-      <c r="E51" s="86">
-        <f>IFERROR(Berechnung!BD8,"-")</f>
-        <v/>
-      </c>
-      <c r="F51" s="86">
-        <f>IFERROR(Berechnung!BC8,"-")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52" ht="22" customHeight="1" s="97">
-      <c r="B52" s="70" t="inlineStr">
-        <is>
-          <t>Q4 2026</t>
-        </is>
-      </c>
-      <c r="C52" s="84">
-        <f>IFERROR(Berechnung!BQ8 &amp; " - " &amp; Berechnung!BR8,"-")</f>
-        <v/>
-      </c>
-      <c r="D52" s="121">
-        <f>IFERROR(Daten!AE8/(Daten!AC8-Daten!AD8),"-")</f>
-        <v/>
-      </c>
-      <c r="E52" s="86">
-        <f>IFERROR(Berechnung!BV8,"-")</f>
-        <v/>
-      </c>
-      <c r="F52" s="86">
-        <f>IFERROR(Berechnung!BU8,"-")</f>
-        <v/>
+      <c r="G6" s="137" t="inlineStr">
+        <is>
+          <t>Laura, Max</t>
+        </is>
+      </c>
+      <c r="H6" s="137" t="inlineStr">
+        <is>
+          <t>#4CAF50</t>
+        </is>
+      </c>
+      <c r="I6" s="137" t="inlineStr">
+        <is>
+          <t>8278b207ba9e80605ae5f1604d696759</t>
+        </is>
+      </c>
+      <c r="J6" s="137" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="137" t="inlineStr">
+        <is>
+          <t>Marleen</t>
+        </is>
+      </c>
+      <c r="B7" s="137" t="n">
+        <v>40</v>
+      </c>
+      <c r="C7" s="137" t="n">
+        <v>80</v>
+      </c>
+      <c r="D7" s="137" t="n">
+        <v>45000</v>
+      </c>
+      <c r="E7" s="137" t="n"/>
+      <c r="F7" s="137" t="inlineStr">
+        <is>
+          <t>Friedrichshain, Charlottenburg, Prenzlauer Berg</t>
+        </is>
+      </c>
+      <c r="G7" s="137" t="inlineStr">
+        <is>
+          <t>Marleen, Luise</t>
+        </is>
+      </c>
+      <c r="H7" s="137" t="inlineStr">
+        <is>
+          <t>#2196F3</t>
+        </is>
+      </c>
+      <c r="I7" s="137" t="inlineStr">
+        <is>
+          <t>0093979f8cf4df0f67ec20b6e35e6beb</t>
+        </is>
+      </c>
+      <c r="J7" s="137" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="137" t="inlineStr">
+        <is>
+          <t>Luise</t>
+        </is>
+      </c>
+      <c r="B8" s="137" t="n">
+        <v>40</v>
+      </c>
+      <c r="C8" s="137" t="n">
+        <v>80</v>
+      </c>
+      <c r="D8" s="137" t="n">
+        <v>40000</v>
+      </c>
+      <c r="E8" s="137" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="F8" s="137" t="inlineStr">
+        <is>
+          <t>Friedrichshain, Charlottenburg, Prenzlauer Berg</t>
+        </is>
+      </c>
+      <c r="G8" s="137" t="inlineStr">
+        <is>
+          <t>Marleen, Luise</t>
+        </is>
+      </c>
+      <c r="H8" s="137" t="inlineStr">
+        <is>
+          <t>#9C27B0</t>
+        </is>
+      </c>
+      <c r="I8" s="137" t="inlineStr">
+        <is>
+          <t>52981192518b734a346928ed713bc015</t>
+        </is>
+      </c>
+      <c r="J8" s="137" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="137" t="inlineStr">
+        <is>
+          <t>Max</t>
+        </is>
+      </c>
+      <c r="B9" s="137" t="n">
+        <v>26</v>
+      </c>
+      <c r="C9" s="137" t="n">
+        <v>65</v>
+      </c>
+      <c r="D9" s="137" t="n">
+        <v>40000</v>
+      </c>
+      <c r="E9" s="137" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="F9" s="137" t="inlineStr">
+        <is>
+          <t>Spandau, Mitte</t>
+        </is>
+      </c>
+      <c r="G9" s="137" t="inlineStr">
+        <is>
+          <t>Laura, Max</t>
+        </is>
+      </c>
+      <c r="H9" s="137" t="inlineStr">
+        <is>
+          <t>#FF9800</t>
+        </is>
+      </c>
+      <c r="I9" s="137" t="inlineStr">
+        <is>
+          <t>5051837ce5b8f243f109306f60136f17</t>
+        </is>
+      </c>
+      <c r="J9" s="137" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="160" t="inlineStr">
+        <is>
+          <t>ℹ️ Bei neuem PM Token erzeugen:</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="161" t="inlineStr">
+        <is>
+          <t>python3 -c "import secrets; print(secrets.token_hex(16))"</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="B39:F39"/>
-    <mergeCell ref="B24:F24"/>
-    <mergeCell ref="B2:F2"/>
-    <mergeCell ref="B38:F38"/>
-    <mergeCell ref="B19:F19"/>
-    <mergeCell ref="B46:F46"/>
-    <mergeCell ref="B1:F1"/>
-    <mergeCell ref="B32:F32"/>
-    <mergeCell ref="B26:F26"/>
-    <mergeCell ref="B13:F13"/>
+  <mergeCells count="3">
+    <mergeCell ref="A12:J12"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A3:J3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Excel-First-Workflow: load_pms_from_excel füllt leere Token/Farbe/Aktiv-Felder automatisch + spiegelt neue PMs in Daten-Tab. add_pm.py entfernt — nicht mehr nötig, Excel ist die einzige Quelle.
</commit_message>
<xml_diff>
--- a/generator/PM_Gehaltsmodell_v18.xlsx
+++ b/generator/PM_Gehaltsmodell_v18.xlsx
@@ -51,7 +51,7 @@
     <numFmt numFmtId="179" formatCode="#,##0.0"/>
     <numFmt numFmtId="180" formatCode="#,##0 €"/>
   </numFmts>
-  <fonts count="50">
+  <fonts count="52">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -357,6 +357,14 @@
       <name val="SF Mono"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001A8A8B"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00666666"/>
+    </font>
   </fonts>
   <fills count="33">
     <fill>
@@ -657,7 +665,7 @@
     <xf numFmtId="43" fontId="24" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="24" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="162">
+  <cellXfs count="164">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1058,6 +1066,8 @@
     </xf>
     <xf numFmtId="0" fontId="48" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="49" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="51" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -10714,7 +10724,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="97" min="1" max="1"/>
@@ -10736,10 +10746,11 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="50" customHeight="1" s="97">
+    <row r="3" ht="60" customHeight="1" s="97">
       <c r="A3" s="137" t="inlineStr">
         <is>
-          <t>Code liest beim Start dieses Sheet, NICHT mehr eine hardcoded Liste. Neuen PM hinzufügen: einfach neue Zeile anhängen, Token via python3 -c "import secrets; print(secrets.token_hex(16))" erzeugen, Daten-Tab Q-Spalten parallel anlegen.</t>
+          <t>Quelle der Wahrheit für die PM-Liste. Code liest beim Start automatisch.
+➜ Neuen PM anlegen: einfach neue Zeile anhängen. Spalte 8 (Farbe), 9 (Token) und 10 (Aktiv) dürfen leer bleiben — werden beim nächsten Dashboard-Lauf automatisch befüllt. Token wird automatisch erzeugt und ins Excel zurückgeschrieben.</t>
         </is>
       </c>
     </row>
@@ -10964,24 +10975,45 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="160" t="inlineStr">
-        <is>
-          <t>ℹ️ Bei neuem PM Token erzeugen:</t>
+      <c r="A11" s="162" t="inlineStr">
+        <is>
+          <t>Auto-Befüllung beim Dashboard-Lauf:</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="161" t="inlineStr">
-        <is>
-          <t>python3 -c "import secrets; print(secrets.token_hex(16))"</t>
+      <c r="A12" s="163" t="inlineStr">
+        <is>
+          <t>• Spalte 8 leer → Default-Farbe #0D595A (Vacura-Teal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="163" t="inlineStr">
+        <is>
+          <t>• Spalte 9 leer → Token wird per secrets.token_hex(16) erzeugt + hier eingetragen</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="163" t="inlineStr">
+        <is>
+          <t>• Spalte 10 leer → Aktiv=Ja angenommen. Auf FALSE setzen um PM zu deaktivieren (z.B. Austritt)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="163" t="inlineStr">
+        <is>
+          <t>• Plus: Daten-Tab Stammdaten-Spalten 1-6 werden parallel gespiegelt, falls dort noch keine Zeile</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A1:J1"/>
     <mergeCell ref="A12:J12"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A3:J3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>